<commit_message>
planilha de autenticação ajuste
</commit_message>
<xml_diff>
--- a/auth.xlsx
+++ b/auth.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\preditiva\PREDITIVA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D2E2F31-6770-4114-8EC5-11C1EA4F289B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50F212AB-D106-42F3-AEFC-FA363EB6E313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{6A472DFD-0E09-42DB-874E-9233951C7FB7}"/>
   </bookViews>
@@ -33,12 +33,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Usuario</t>
   </si>
   <si>
     <t>Senha</t>
+  </si>
+  <si>
+    <t>admin</t>
   </si>
 </sst>
 </file>
@@ -426,7 +429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13F37F4D-7674-4A32-8889-363E089154EA}">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -445,8 +448,8 @@
         <v>11</v>
       </c>
       <c r="B2" t="str">
-        <f>A2 &amp; " - kidy@2025"</f>
-        <v>11 - kidy@2025</v>
+        <f>A2&amp;"kidy@2025"</f>
+        <v>11kidy@2025</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -454,8 +457,8 @@
         <v>15</v>
       </c>
       <c r="B3" t="str">
-        <f t="shared" ref="B3:B52" si="0">A3 &amp; " - kidy@2025"</f>
-        <v>15 - kidy@2025</v>
+        <f t="shared" ref="B3:B52" si="0">A3&amp;"kidy@2025"</f>
+        <v>15kidy@2025</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -464,7 +467,7 @@
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
-        <v>19 - kidy@2025</v>
+        <v>19kidy@2025</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -473,7 +476,7 @@
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
-        <v>23 - kidy@2025</v>
+        <v>23kidy@2025</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -482,7 +485,7 @@
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
-        <v>31 - kidy@2025</v>
+        <v>31kidy@2025</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -491,7 +494,7 @@
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
-        <v>34 - kidy@2025</v>
+        <v>34kidy@2025</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -500,7 +503,7 @@
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
-        <v>38 - kidy@2025</v>
+        <v>38kidy@2025</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -509,7 +512,7 @@
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
-        <v>39 - kidy@2025</v>
+        <v>39kidy@2025</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -518,7 +521,7 @@
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
-        <v>41 - kidy@2025</v>
+        <v>41kidy@2025</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -527,7 +530,7 @@
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
-        <v>45 - kidy@2025</v>
+        <v>45kidy@2025</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -536,7 +539,7 @@
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
-        <v>46 - kidy@2025</v>
+        <v>46kidy@2025</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -545,7 +548,7 @@
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
-        <v>53 - kidy@2025</v>
+        <v>53kidy@2025</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -554,7 +557,7 @@
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
-        <v>61 - kidy@2025</v>
+        <v>61kidy@2025</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -563,7 +566,7 @@
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
-        <v>65 - kidy@2025</v>
+        <v>65kidy@2025</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -572,7 +575,7 @@
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
-        <v>74 - kidy@2025</v>
+        <v>74kidy@2025</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -581,7 +584,7 @@
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
-        <v>93 - kidy@2025</v>
+        <v>93kidy@2025</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -590,7 +593,7 @@
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
-        <v>143 - kidy@2025</v>
+        <v>143kidy@2025</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -599,7 +602,7 @@
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
-        <v>167 - kidy@2025</v>
+        <v>167kidy@2025</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -608,7 +611,7 @@
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
-        <v>371 - kidy@2025</v>
+        <v>371kidy@2025</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -617,7 +620,7 @@
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
-        <v>178 - kidy@2025</v>
+        <v>178kidy@2025</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -626,7 +629,7 @@
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
-        <v>187 - kidy@2025</v>
+        <v>187kidy@2025</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -635,7 +638,7 @@
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
-        <v>194 - kidy@2025</v>
+        <v>194kidy@2025</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -644,7 +647,7 @@
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
-        <v>197 - kidy@2025</v>
+        <v>197kidy@2025</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -653,7 +656,7 @@
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
-        <v>208 - kidy@2025</v>
+        <v>208kidy@2025</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -662,7 +665,7 @@
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
-        <v>217 - kidy@2025</v>
+        <v>217kidy@2025</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -671,7 +674,7 @@
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
-        <v>218 - kidy@2025</v>
+        <v>218kidy@2025</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -680,7 +683,7 @@
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
-        <v>231 - kidy@2025</v>
+        <v>231kidy@2025</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -689,7 +692,7 @@
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
-        <v>232 - kidy@2025</v>
+        <v>232kidy@2025</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -698,7 +701,7 @@
       </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
-        <v>240 - kidy@2025</v>
+        <v>240kidy@2025</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -707,7 +710,7 @@
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
-        <v>248 - kidy@2025</v>
+        <v>248kidy@2025</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -716,7 +719,7 @@
       </c>
       <c r="B32" t="str">
         <f t="shared" si="0"/>
-        <v>261 - kidy@2025</v>
+        <v>261kidy@2025</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -725,7 +728,7 @@
       </c>
       <c r="B33" t="str">
         <f t="shared" si="0"/>
-        <v>266 - kidy@2025</v>
+        <v>266kidy@2025</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -734,7 +737,7 @@
       </c>
       <c r="B34" t="str">
         <f t="shared" si="0"/>
-        <v>267 - kidy@2025</v>
+        <v>267kidy@2025</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +746,7 @@
       </c>
       <c r="B35" t="str">
         <f t="shared" si="0"/>
-        <v>270 - kidy@2025</v>
+        <v>270kidy@2025</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -752,7 +755,7 @@
       </c>
       <c r="B36" t="str">
         <f t="shared" si="0"/>
-        <v>273 - kidy@2025</v>
+        <v>273kidy@2025</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -761,7 +764,7 @@
       </c>
       <c r="B37" t="str">
         <f t="shared" si="0"/>
-        <v>282 - kidy@2025</v>
+        <v>282kidy@2025</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -770,7 +773,7 @@
       </c>
       <c r="B38" t="str">
         <f t="shared" si="0"/>
-        <v>291 - kidy@2025</v>
+        <v>291kidy@2025</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -779,7 +782,7 @@
       </c>
       <c r="B39" t="str">
         <f t="shared" si="0"/>
-        <v>292 - kidy@2025</v>
+        <v>292kidy@2025</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -788,7 +791,7 @@
       </c>
       <c r="B40" t="str">
         <f t="shared" si="0"/>
-        <v>294 - kidy@2025</v>
+        <v>294kidy@2025</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -797,7 +800,7 @@
       </c>
       <c r="B41" t="str">
         <f t="shared" si="0"/>
-        <v>296 - kidy@2025</v>
+        <v>296kidy@2025</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -806,7 +809,7 @@
       </c>
       <c r="B42" t="str">
         <f t="shared" si="0"/>
-        <v>297 - kidy@2025</v>
+        <v>297kidy@2025</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -815,7 +818,7 @@
       </c>
       <c r="B43" t="str">
         <f t="shared" si="0"/>
-        <v>298 - kidy@2025</v>
+        <v>298kidy@2025</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -824,7 +827,7 @@
       </c>
       <c r="B44" t="str">
         <f t="shared" si="0"/>
-        <v>299 - kidy@2025</v>
+        <v>299kidy@2025</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -833,7 +836,7 @@
       </c>
       <c r="B45" t="str">
         <f t="shared" si="0"/>
-        <v>301 - kidy@2025</v>
+        <v>301kidy@2025</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -842,7 +845,7 @@
       </c>
       <c r="B46" t="str">
         <f t="shared" si="0"/>
-        <v>302 - kidy@2025</v>
+        <v>302kidy@2025</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -851,7 +854,7 @@
       </c>
       <c r="B47" t="str">
         <f t="shared" si="0"/>
-        <v>308 - kidy@2025</v>
+        <v>308kidy@2025</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -860,7 +863,7 @@
       </c>
       <c r="B48" t="str">
         <f t="shared" si="0"/>
-        <v>311 - kidy@2025</v>
+        <v>311kidy@2025</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -869,7 +872,7 @@
       </c>
       <c r="B49" t="str">
         <f t="shared" si="0"/>
-        <v>315 - kidy@2025</v>
+        <v>315kidy@2025</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -878,7 +881,7 @@
       </c>
       <c r="B50" t="str">
         <f t="shared" si="0"/>
-        <v>316 - kidy@2025</v>
+        <v>316kidy@2025</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -887,7 +890,7 @@
       </c>
       <c r="B51" t="str">
         <f t="shared" si="0"/>
-        <v>317 - kidy@2025</v>
+        <v>317kidy@2025</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -896,7 +899,15 @@
       </c>
       <c r="B52" t="str">
         <f t="shared" si="0"/>
-        <v>320 - kidy@2025</v>
+        <v>320kidy@2025</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>2</v>
+      </c>
+      <c r="B53">
+        <v>497980</v>
       </c>
     </row>
   </sheetData>

</xml_diff>